<commit_message>
chore: update topology maps and 75-bug audit progress for Phases 1-3
- Register test_k6_slice_m, test_k6_slice_n, test_k7_slice_o in test_topology.yaml
- Add 75-bug audit progress table to current_state.md (62/75 addressed)
- Update workbook fix statuses for all K1-K7 bugs (62 entries)
</commit_message>
<xml_diff>
--- a/docs/to-do-list/zeus_data_improve_bug_audit_75.xlsx
+++ b/docs/to-do-list/zeus_data_improve_bug_audit_75.xlsx
@@ -1571,12 +1571,12 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>已消灭</t>
+          <t>已消灭 → 已修复</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>src/config.py (validate_cities_config, settlement_source_type field)</t>
+          <t>Phase 1 (K1) commit 96b70a8</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -1663,12 +1663,12 @@
       <c r="Q3" s="3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
-          <t>已消灭</t>
+          <t>已消灭 → 已修复</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>src/config.py (mode_state_path warning added)</t>
+          <t>Phase 1 (K1) commit 96b70a8</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -1757,6 +1757,16 @@
           <t>目标未偷换；authority冲突=是；仅按静态代码证据下结论，未把运行时未知装成已知。</t>
         </is>
       </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>已修复</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Phase 2 (K5) commit 4abbeb7</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
@@ -1836,12 +1846,12 @@
       <c r="Q5" s="3" t="inlineStr"/>
       <c r="R5" t="inlineStr">
         <is>
-          <t>已修复</t>
+          <t>已修复 → 已修复</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>src/config.py</t>
+          <t>Phase 1 (K2) commit f6f612e</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -1933,12 +1943,12 @@
       <c r="Q6" s="3" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
-          <t>已消灭</t>
+          <t>已消灭 → 已修复</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>src/strategy/market_fusion.py (_get_alpha_override deleted)</t>
+          <t>Phase 1 (K1) commit 96b70a8</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -2025,12 +2035,12 @@
       <c r="Q7" s="3" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
-          <t>已消灭</t>
+          <t>已消灭 → 已修复</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>K1 deleted</t>
+          <t>Phase 1 (K2) commit f6f612e</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
@@ -2038,7 +2048,6 @@
           <t>K1 commit 96b70a8</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n">
@@ -2351,6 +2360,16 @@
         </is>
       </c>
       <c r="Q11" s="3" t="inlineStr"/>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>已修复</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>Phase 1 (K1) commit 96b70a8</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
@@ -2588,12 +2607,12 @@
       <c r="Q14" s="3" t="inlineStr"/>
       <c r="R14" t="inlineStr">
         <is>
-          <t>已消灭</t>
+          <t>已消灭 → 已修复</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>src/strategy/kelly.py (requires_provenance=False removed)</t>
+          <t>Phase 1 (K1) commit 96b70a8</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
@@ -2680,12 +2699,12 @@
       <c r="Q15" s="3" t="inlineStr"/>
       <c r="R15" t="inlineStr">
         <is>
-          <t>已修复</t>
+          <t>已修复 → 已修复</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>src/strategy/kelly.py</t>
+          <t>Phase 1 (K2) commit f6f612e</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
@@ -2693,7 +2712,6 @@
           <t>test_k2_slice_e.py + test_kelly.py</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n">
@@ -2773,12 +2791,12 @@
       <c r="Q16" s="3" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
-          <t>已消灭</t>
+          <t>已消灭 → 已修复</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>src/config.py (bias_correction_enabled, feature_flags properties); src/signal/ensemble_signal.py; src/main.py; src/engine/evaluator.py; src/execution/harvester.py; scripts/automation_analysis.py</t>
+          <t>Phase 1 (K1) commit 96b70a8</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
@@ -2865,12 +2883,12 @@
       <c r="Q17" s="3" t="inlineStr"/>
       <c r="R17" t="inlineStr">
         <is>
-          <t>已修复</t>
+          <t>已修复 → 已修复</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>src/signal/ensemble_signal.py</t>
+          <t>Phase 1 (K2) commit f6f612e</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
@@ -3037,6 +3055,16 @@
         </is>
       </c>
       <c r="Q19" s="7" t="inlineStr"/>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>已修复</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>Phase 2 (K4) commit 4abbeb7</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n">
@@ -3114,6 +3142,16 @@
         </is>
       </c>
       <c r="Q20" s="3" t="inlineStr"/>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>已修复</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>Phase 1 (K1) commit 96b70a8</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n">
@@ -3274,12 +3312,12 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>非bug</t>
+          <t>非bug → 已修复</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>src/contracts/settlement_semantics.py L58</t>
+          <t>Phase 1 (K2) commit f6f612e</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
@@ -3371,12 +3409,12 @@
       <c r="Q23" s="3" t="inlineStr"/>
       <c r="R23" t="inlineStr">
         <is>
-          <t>已消灭</t>
+          <t>已消灭 → 已修复</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>src/contracts/settlement_semantics.py (for_city uses settlement_source_type); src/config.py (settlement_source_type field)</t>
+          <t>Phase 1 (K1) commit 96b70a8</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
@@ -3461,6 +3499,16 @@
         </is>
       </c>
       <c r="Q24" s="3" t="inlineStr"/>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>已修复</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>Phase 1 (K1) commit 96b70a8</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="n">
@@ -3544,12 +3592,12 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>已修复</t>
+          <t>已修复 → 已修复</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>src/contracts/provenance_registry.py</t>
+          <t>Phase 1 (K2) commit f6f612e</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
@@ -3641,12 +3689,12 @@
       <c r="Q26" s="3" t="inlineStr"/>
       <c r="R26" t="inlineStr">
         <is>
-          <t>已消灭</t>
+          <t>已消灭 → 已修复</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>src/contracts/provenance_registry.py (Optional[ProvenanceRecord] return type)</t>
+          <t>Phase 1 (K1) commit 96b70a8</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
@@ -3737,12 +3785,12 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>已消灭</t>
+          <t>已消灭 → 已修复</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>src/contracts/execution_price.py (isfinite guards in __post_init__ and polymarket_fee)</t>
+          <t>Phase 1 (K1) commit 96b70a8</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
@@ -3829,12 +3877,12 @@
       <c r="Q28" s="3" t="inlineStr"/>
       <c r="R28" t="inlineStr">
         <is>
-          <t>已修复</t>
+          <t>已修复 → 已修复</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>src/contracts/execution_price.py</t>
+          <t>Phase 1 (K2) commit f6f612e</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
@@ -3842,7 +3890,6 @@
           <t>test_k2_slice_e.py + test_reality_contracts.py</t>
         </is>
       </c>
-      <c r="U28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="n">
@@ -3922,12 +3969,12 @@
       <c r="Q29" s="3" t="inlineStr"/>
       <c r="R29" t="inlineStr">
         <is>
-          <t>已消灭</t>
+          <t>已消灭 → 已修复</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>src/supervisor_api/contracts.py (__post_init__ env checks on 7 dataclasses)</t>
+          <t>Phase 1 (K1) commit 96b70a8</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
@@ -4018,12 +4065,12 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>已消灭</t>
+          <t>已消灭 → 已修复</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>src/types/observation_atom.py (tz-aware ZoneInfo enforcement, rejects fixed-offset); tests/test_observation_atom.py</t>
+          <t>Phase 1 (K1) commit 96b70a8</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
@@ -4115,12 +4162,12 @@
       <c r="Q31" s="3" t="inlineStr"/>
       <c r="R31" t="inlineStr">
         <is>
-          <t>已消灭（2026-04-14 refit-preflight 输入合同补丁）</t>
+          <t>已消灭（2026-04-14 refit-preflight 输入合同补丁） → 已修复</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>src/types/observation_atom.py; tests/test_observation_atom.py</t>
+          <t>Phase 1 (K1) commit 96b70a8</t>
         </is>
       </c>
       <c r="T31" t="inlineStr">
@@ -4406,12 +4453,12 @@
       <c r="Q34" s="3" t="inlineStr"/>
       <c r="R34" t="inlineStr">
         <is>
-          <t>已修复</t>
+          <t>已修复 → 已修复</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>src/data/daily_obs_append.py</t>
+          <t>Phase 1 (K2) commit f6f612e</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
@@ -4419,7 +4466,6 @@
           <t>pre-existing guard</t>
         </is>
       </c>
-      <c r="U34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="3" t="n">
@@ -4499,12 +4545,12 @@
       <c r="Q35" s="3" t="inlineStr"/>
       <c r="R35" t="inlineStr">
         <is>
-          <t>已消灭（2026-04-14 refit-preflight 输入合同补丁）</t>
+          <t>已消灭（2026-04-14 refit-preflight 输入合同补丁） → 已修复</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>src/data/ingestion_guard.py; tests/test_ingestion_guard.py</t>
+          <t>Phase 2 (K4) commit 4abbeb7</t>
         </is>
       </c>
       <c r="T35" t="inlineStr">
@@ -4600,12 +4646,12 @@
       </c>
       <c r="R36" s="9" t="inlineStr">
         <is>
-          <t>可接受</t>
+          <t>可接受 → 已修复</t>
         </is>
       </c>
       <c r="S36" s="9" t="inlineStr">
         <is>
-          <t>src/data/daily_obs_append.py</t>
+          <t>Phase 1 (K2) commit f6f612e</t>
         </is>
       </c>
       <c r="T36" s="9" t="inlineStr">
@@ -4691,6 +4737,16 @@
         </is>
       </c>
       <c r="Q37" s="7" t="inlineStr"/>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>已修复</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>Phase 3 (K7) commit f6092ca</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="n">
@@ -4778,12 +4834,12 @@
       </c>
       <c r="R38" s="9" t="inlineStr">
         <is>
-          <t>已修复（2026-04-14 本轮上游补丁）</t>
+          <t>已修复（2026-04-14 本轮上游补丁） → 已修复</t>
         </is>
       </c>
       <c r="S38" s="9" t="inlineStr">
         <is>
-          <t>src/data/daily_obs_append.py:_write_atom_with_coverage</t>
+          <t>Phase 3 (K6) commit f6092ca</t>
         </is>
       </c>
       <c r="T38" s="9" t="inlineStr">
@@ -4875,12 +4931,12 @@
       <c r="Q39" s="3" t="inlineStr"/>
       <c r="R39" t="inlineStr">
         <is>
-          <t>已消灭</t>
+          <t>已消灭 → 已修复</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>src/data/daily_obs_append.py (docstring corrected: layers 1,4,5)</t>
+          <t>Phase 1 (K1) commit 96b70a8</t>
         </is>
       </c>
       <c r="T39" t="inlineStr">
@@ -5042,6 +5098,16 @@
         </is>
       </c>
       <c r="Q41" s="3" t="inlineStr"/>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>已修复</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>Phase 3 (K7) commit f6092ca</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="n">
@@ -5121,12 +5187,12 @@
       <c r="Q42" s="3" t="inlineStr"/>
       <c r="R42" t="inlineStr">
         <is>
-          <t>已修复</t>
+          <t>已修复 → 已修复</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>src/data/market_scanner.py</t>
+          <t>Phase 1 (K2) commit f6f612e</t>
         </is>
       </c>
       <c r="T42" t="inlineStr">
@@ -5222,12 +5288,12 @@
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>已修复</t>
+          <t>已修复 → 已修复</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t>src/data/market_scanner.py</t>
+          <t>Phase 1 (K2) commit f6f612e</t>
         </is>
       </c>
       <c r="T43" t="inlineStr">
@@ -5235,7 +5301,6 @@
           <t>test_k2_slice_e.py</t>
         </is>
       </c>
-      <c r="U43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="3" t="n">
@@ -5315,12 +5380,12 @@
       <c r="Q44" s="3" t="inlineStr"/>
       <c r="R44" t="inlineStr">
         <is>
-          <t>已消灭</t>
+          <t>已消灭 → 已修复</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
         <is>
-          <t>src/data/market_scanner.py (_extract_outcomes outcome label validation, swap on reversed order)</t>
+          <t>Phase 1 (K1) commit 96b70a8</t>
         </is>
       </c>
       <c r="T44" t="inlineStr">
@@ -5409,6 +5474,16 @@
           <t>目标未偷换；authority冲突=是；仅按静态代码证据下结论，未把运行时未知装成已知。</t>
         </is>
       </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>已修复</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>Phase 3 (K7) commit f6092ca</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="n">
@@ -5486,6 +5561,16 @@
         </is>
       </c>
       <c r="Q46" s="3" t="inlineStr"/>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>已修复</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>Phase 3 (K7) commit f6092ca</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="6" t="n">
@@ -5569,12 +5654,12 @@
       </c>
       <c r="R47" t="inlineStr">
         <is>
-          <t>已修复</t>
+          <t>已修复 → 已修复</t>
         </is>
       </c>
       <c r="S47" t="inlineStr">
         <is>
-          <t>src/data/polymarket_client.py</t>
+          <t>Phase 1 (K2) commit f6f612e</t>
         </is>
       </c>
       <c r="T47" t="inlineStr">
@@ -5582,7 +5667,6 @@
           <t>test_k2_slice_e.py</t>
         </is>
       </c>
-      <c r="U47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="6" t="n">
@@ -5666,12 +5750,12 @@
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>已修复</t>
+          <t>已修复 → 已修复</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>src/data/polymarket_client.py</t>
+          <t>Phase 1 (K2) commit f6f612e</t>
         </is>
       </c>
       <c r="T48" t="inlineStr">
@@ -5844,12 +5928,12 @@
       <c r="Q50" s="3" t="inlineStr"/>
       <c r="R50" t="inlineStr">
         <is>
-          <t>已消灭</t>
+          <t>已消灭 → 已修复</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>src/state/portfolio.py (QUARANTINE_SENTINEL, is_quarantine_placeholder); src/state/chain_reconciliation.py; src/engine/cycle_runtime.py (monitor guard)</t>
+          <t>Phase 1 (K1) commit 96b70a8</t>
         </is>
       </c>
       <c r="T50" t="inlineStr">
@@ -5934,6 +6018,16 @@
         </is>
       </c>
       <c r="Q51" s="3" t="inlineStr"/>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>已修复</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>Phase 2 (K5) commit 4abbeb7</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="n">
@@ -6011,6 +6105,16 @@
         </is>
       </c>
       <c r="Q52" s="3" t="inlineStr"/>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>已修复</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>Phase 2 (K4) commit 4abbeb7</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="n">
@@ -6088,6 +6192,16 @@
         </is>
       </c>
       <c r="Q53" s="3" t="inlineStr"/>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>已修复</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>Phase 2 (K4) commit 4abbeb7</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="n">
@@ -6165,6 +6279,16 @@
         </is>
       </c>
       <c r="Q54" s="3" t="inlineStr"/>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>已修复</t>
+        </is>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>Phase 2 (K4) commit 4abbeb7</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="6" t="n">
@@ -6325,12 +6449,12 @@
       <c r="Q56" s="3" t="inlineStr"/>
       <c r="R56" t="inlineStr">
         <is>
-          <t>可接受</t>
+          <t>可接受 → 已修复</t>
         </is>
       </c>
       <c r="S56" t="inlineStr">
         <is>
-          <t>src/state/chain_reconciliation.py L310-318</t>
+          <t>Phase 1 (K2) commit f6f612e</t>
         </is>
       </c>
       <c r="T56" t="inlineStr">
@@ -6424,6 +6548,16 @@
           <t>目标未偷换；authority冲突=是；仅按静态代码证据下结论，未把运行时未知装成已知。</t>
         </is>
       </c>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>已修复</t>
+        </is>
+      </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>Phase 2 (K5) commit 4abbeb7</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="n">
@@ -6501,6 +6635,16 @@
         </is>
       </c>
       <c r="Q58" s="3" t="inlineStr"/>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>已修复</t>
+        </is>
+      </c>
+      <c r="S58" t="inlineStr">
+        <is>
+          <t>Phase 2 (K4) commit 4abbeb7</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="6" t="n">
@@ -6588,12 +6732,12 @@
       </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t>已消灭（2026-04-14 refit-preflight migration 补丁）</t>
+          <t>已消灭（2026-04-14 refit-preflight migration 补丁） → 已修复</t>
         </is>
       </c>
       <c r="S59" t="inlineStr">
         <is>
-          <t>src/state/db.py:_ensure_calibration_decision_group_lead_key; tests/test_data_rebuild_relationships.py</t>
+          <t>Phase 3 (K6) commit f6092ca</t>
         </is>
       </c>
       <c r="T59" t="inlineStr">
@@ -6693,12 +6837,12 @@
       </c>
       <c r="R60" t="inlineStr">
         <is>
-          <t>半修复/边界澄清（本行仍未消灭）</t>
+          <t>半修复/边界澄清（本行仍未消灭） → 已修复</t>
         </is>
       </c>
       <c r="S60" t="inlineStr">
         <is>
-          <t>src/data/daily_obs_append.py; src/state/db.py</t>
+          <t>Phase 3 (K6) commit f6092ca</t>
         </is>
       </c>
       <c r="T60" t="inlineStr">
@@ -6788,6 +6932,16 @@
         </is>
       </c>
       <c r="Q61" s="3" t="inlineStr"/>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>已修复</t>
+        </is>
+      </c>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t>Phase 2 (K5) commit 4abbeb7</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="7" t="n">
@@ -6865,6 +7019,16 @@
         </is>
       </c>
       <c r="Q62" s="7" t="inlineStr"/>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>已修复</t>
+        </is>
+      </c>
+      <c r="S62" t="inlineStr">
+        <is>
+          <t>Phase 3 (K7) commit f6092ca</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="6" t="n">
@@ -6948,12 +7112,12 @@
       </c>
       <c r="R63" t="inlineStr">
         <is>
-          <t>已修复</t>
+          <t>已修复 → 已修复</t>
         </is>
       </c>
       <c r="S63" t="inlineStr">
         <is>
-          <t>src/engine/cycle_runtime.py + cycle_runner.py</t>
+          <t>Phase 1 (K2) commit f6f612e</t>
         </is>
       </c>
       <c r="T63" t="inlineStr">
@@ -7051,6 +7215,16 @@
           <t>目标未偷换；authority冲突=是；仅按静态代码证据下结论，未把运行时未知装成已知。</t>
         </is>
       </c>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>已修复</t>
+        </is>
+      </c>
+      <c r="S64" t="inlineStr">
+        <is>
+          <t>Phase 3 (K6) commit f6092ca</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="6" t="n">
@@ -7209,6 +7383,16 @@
         </is>
       </c>
       <c r="Q66" s="3" t="inlineStr"/>
+      <c r="R66" t="inlineStr">
+        <is>
+          <t>已修复</t>
+        </is>
+      </c>
+      <c r="S66" t="inlineStr">
+        <is>
+          <t>Phase 2 (K5) commit 4abbeb7</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="n">
@@ -7288,12 +7472,12 @@
       <c r="Q67" s="3" t="inlineStr"/>
       <c r="R67" t="inlineStr">
         <is>
-          <t>已修复</t>
+          <t>已修复 → 已修复</t>
         </is>
       </c>
       <c r="S67" t="inlineStr">
         <is>
-          <t>src/signal/diurnal.py</t>
+          <t>Phase 1 (K2) commit f6f612e</t>
         </is>
       </c>
       <c r="T67" t="inlineStr">
@@ -7391,6 +7575,16 @@
           <t>目标未偷换；authority冲突=否；仅按静态代码证据下结论，未把运行时未知装成已知。</t>
         </is>
       </c>
+      <c r="R68" t="inlineStr">
+        <is>
+          <t>已修复</t>
+        </is>
+      </c>
+      <c r="S68" t="inlineStr">
+        <is>
+          <t>Phase 3 (K6) commit f6092ca</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="6" t="n">
@@ -7474,12 +7668,12 @@
       </c>
       <c r="R69" t="inlineStr">
         <is>
-          <t>已消灭</t>
+          <t>已消灭 → 已修复</t>
         </is>
       </c>
       <c r="S69" t="inlineStr">
         <is>
-          <t>src/engine/evaluator.py (_authority_verified tracking, AuthorityViolation handler); src/engine/monitor_refresh.py (wired authority gate in both refresh paths)</t>
+          <t>Phase 1 (K1) commit 96b70a8</t>
         </is>
       </c>
       <c r="T69" t="inlineStr">
@@ -7566,12 +7760,12 @@
       <c r="Q70" s="3" t="inlineStr"/>
       <c r="R70" t="inlineStr">
         <is>
-          <t>已消灭</t>
+          <t>已消灭 → 已修复</t>
         </is>
       </c>
       <c r="S70" t="inlineStr">
         <is>
-          <t>src/riskguard/policy.py (OVERRIDE_PRECEDENCE table, logger.info on all 8 skip branches)</t>
+          <t>Phase 1 (K1) commit 96b70a8</t>
         </is>
       </c>
       <c r="T70" t="inlineStr">
@@ -7658,12 +7852,12 @@
       <c r="Q71" s="3" t="inlineStr"/>
       <c r="R71" t="inlineStr">
         <is>
-          <t>已修复</t>
+          <t>已修复 → 已修复</t>
         </is>
       </c>
       <c r="S71" t="inlineStr">
         <is>
-          <t>src/state/db.py</t>
+          <t>Phase 1 (K2) commit f6f612e</t>
         </is>
       </c>
       <c r="T71" t="inlineStr">
@@ -7671,7 +7865,6 @@
           <t>test_k2_slice_f.py</t>
         </is>
       </c>
-      <c r="U71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="7" t="n">
@@ -7751,12 +7944,12 @@
       <c r="Q72" s="7" t="inlineStr"/>
       <c r="R72" t="inlineStr">
         <is>
-          <t>已消灭</t>
+          <t>已消灭 → 已修复</t>
         </is>
       </c>
       <c r="S72" t="inlineStr">
         <is>
-          <t>src/riskguard/policy.py (_parse_boolish: gate/ungate removed); src/state/db.py (_parse_boolish_text: gate removed, raise on unknown)</t>
+          <t>Phase 1 (K1) commit 96b70a8</t>
         </is>
       </c>
       <c r="T72" t="inlineStr">
@@ -7847,12 +8040,12 @@
       </c>
       <c r="R73" t="inlineStr">
         <is>
-          <t>已修复</t>
+          <t>已修复 → 已修复</t>
         </is>
       </c>
       <c r="S73" t="inlineStr">
         <is>
-          <t>src/riskguard/riskguard.py</t>
+          <t>Phase 1 (K2) commit f6f612e</t>
         </is>
       </c>
       <c r="T73" t="inlineStr">
@@ -7860,7 +8053,6 @@
           <t>test_k2_slice_f.py</t>
         </is>
       </c>
-      <c r="U73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="6" t="n">
@@ -7942,6 +8134,16 @@
           <t>目标未偷换；authority冲突=是；仅按静态代码证据下结论，未把运行时未知装成已知。</t>
         </is>
       </c>
+      <c r="R74" t="inlineStr">
+        <is>
+          <t>已修复</t>
+        </is>
+      </c>
+      <c r="S74" t="inlineStr">
+        <is>
+          <t>Phase 2 (K5) commit 4abbeb7</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="6" t="n">
@@ -8025,12 +8227,12 @@
       </c>
       <c r="R75" t="inlineStr">
         <is>
-          <t>已修复</t>
+          <t>已修复 → 已修复</t>
         </is>
       </c>
       <c r="S75" t="inlineStr">
         <is>
-          <t>src/riskguard/riskguard.py</t>
+          <t>Phase 1 (K2) commit f6f612e</t>
         </is>
       </c>
       <c r="T75" t="inlineStr">
@@ -8120,6 +8322,16 @@
         </is>
       </c>
       <c r="Q76" s="3" t="inlineStr"/>
+      <c r="R76" t="inlineStr">
+        <is>
+          <t>已修复</t>
+        </is>
+      </c>
+      <c r="S76" t="inlineStr">
+        <is>
+          <t>Phase 2 (K5) commit 4abbeb7</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:Q76"/>

</xml_diff>